<commit_message>
definir origem - ok
</commit_message>
<xml_diff>
--- a/contatos.xlsx
+++ b/contatos.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="20">
   <si>
     <t>CONTATO</t>
   </si>
@@ -42,13 +42,16 @@
     <t>29-01</t>
   </si>
   <si>
-    <t>TELEFONE</t>
-  </si>
-  <si>
-    <t>EMAIL</t>
-  </si>
-  <si>
-    <t>ANIVERSARIO/VENCIMENTO</t>
+    <t>nome</t>
+  </si>
+  <si>
+    <t>telefone</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>aniversario</t>
   </si>
   <si>
     <t>BOB1</t>
@@ -521,31 +524,31 @@
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="8" t="s">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E1" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B2" s="4">
         <v>21997633265</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E2" s="3"/>
     </row>
@@ -557,25 +560,25 @@
         <v>2137074557</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E3" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B4" s="4">
-        <v>2121212121</v>
+        <v>21997633265</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E4" s="10"/>
     </row>

</xml_diff>